<commit_message>
Add Excel context and row density checks
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/context_workbook.xlsx
+++ b/tests/fixtures/excel/context_workbook.xlsx
@@ -470,33 +470,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Tag assignments</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C1">
-        <f>B2+1</f>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Calculated total</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Calming</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <f>B4+1</f>
         <v/>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Calming</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>